<commit_message>
feat: Railway-Export und Finance-Status nachziehen
</commit_message>
<xml_diff>
--- a/TrafagSalesExporter/docs/Issue_Log_Ingo_2026-08-12.xlsx
+++ b/TrafagSalesExporter/docs/Issue_Log_Ingo_2026-08-12.xlsx
@@ -132,142 +132,145 @@
     <x:t>Daten für TR ES Jan bis Mai 2026 fehlen</x:t>
   </x:si>
   <x:si>
+    <x:t>Mittel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Keine, Lücke ist geschlossen. Restliche Buchungsdatum-Lücke ab Juni ist unter ISS-004.2 erfasst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SageSpainExportPackage/; Spain_Sales_range_20260528_to_20260603.csv</x:t>
+  </x:si>
+  <x:si>
+    <x:t>28.07.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>STATUS KORRIGIERT: stand als "Warten auf andere" mit Mail an Rohail. Es muss aber niemand antworten, denn die Sage-Export-SQL ist unsere und liegt in SageSpainExportPackage. Owner ist damit Ingo. Am 12.08.2026 unverändert bestätigt: Januar bis April 0 Zeilen, Mai nur 35, danach normal mit Juni 542 und Juli 503. 2025 ist über alle zwölf Monate vollständig. NACHTRAG 17.08.2026: der Range-Export Januar bis Mai 2026 ist lokal gelaufen, hat 1'571 Zeilen mit 100 % gefülltem PostingDate geliefert und ist per rclone nach Import/Finance/Spanien hochgeladen. NACHTRAG 18.08.2026: Import bestätigt und gegengemessen. TRES steht bei 7'220 Zeilen statt 5'712 am 12.08., nach InvoiceDate durchgehend ohne Nullmonat von Januar 2025 bis Juli 2026. Lücke damit geschlossen.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISS-001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TR AT und CH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Daten scheinen ab Mitte April nur noch vereinzelt geladen zu werden</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Beim nächsten Monatswechsel einmal gegenprüfen, dass der SAP-Batchjob weiterhin läuft</x:t>
+  </x:si>
+  <x:si>
+    <x:t>.tmp_tools/OdataProbe; docs/FINANCE_CHAT_2026_LUECKE_ROOTCAUSE_2026-07-28.md</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Zwei Stufen, beide erledigt. Erstens die Ursache von Juli: das Dashboard las das TEST-System T76 statt P76; Sites.SapServiceUrl steht inzwischen auf travp762, damit ist auch der frühere Punkt "Quelle umstellen" durch, und 2025 ist mit 30'642 Zeilen in beiden Systemen vollständig. Zweitens ein Folgeproblem, das darunter lag und im alten Log fehlte: von 31.07. bis 12.08. kamen für AT und CH KEINE neuen Zeilen, weil der SAP-Report Z_TRAFAG_DACH_EXPORT nur manuell lief. Ingo hat den Batchjob ZSCHWEIZ am 12.08.2026 auf täglich gestellt, und der Gesamtexport all8.xlsx von 14:39 belegt die Wirkung am selben Tag: CH 48'276 statt 47'142 Zeilen, AT 1'839 statt 1'790, August 2026 erstmals vorhanden, letzter Beleg 12.08. Der Wert liegt im vorher berechneten Fenster, 2025 ist erhalten und 2026 wurde ersetzt statt verdoppelt.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISS-001.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Datenzufluss TR FR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>B1 Frankreich enthält seit dem 30.07.2026 keine Rechnung mehr</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Warten auf andere</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Frankreich / Ingo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Frankreich gezielt fragen, warum seit dem 30.07. weder geliefert noch fakturiert wird, obwohl Aufträge und Wareneingänge weiterlaufen, und wann der Rückstand nachgebucht wird</x:t>
+  </x:si>
+  <x:si>
+    <x:t>.tmp_tools/HanaQ gegen FR01_P mit OINV, ORIN, ODLN, ORDR, ODRF (read-only, 12.08.2026)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Antwort aus Frankreich</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NEU AUFGENOMMEN, im alten Log nicht enthalten. Direkt in der Quelle geprüft: Rechnungen OINV letzter 30.07., Lieferscheine ODLN letzter 30.07., Gutschriften ORIN keine seit dem 25.07., Aufträge ORDR letzter 07.08., Entwürfe ODRF 12 Stück am 11.08. und alle vom Typ 20, also Wareneingänge zu Bestellungen. Frankreich arbeitet also weiter, nimmt Aufträge an und empfängt Ware, liefert und fakturiert aber nicht. Warenausgang und Faktura enden am exakt selben Tag, das deutet auf eine Betriebsschliessung oder eine Sperre im Ausgangsprozess, nicht auf ein Systemproblem. Saisonalität allein erklärt es nicht, im August 2025 gab es 99 Zeilen. Eine zweite Firmendatenbank aus dem B1-Upgrade ist ausgeschlossen, SYS.SCHEMAS kennt nur FR01_P. Die täglich frischen TRFR-Dateien in SharePoint sind UNSERE Exportausgaben, keine Lieferung aus Frankreich, und enthalten unverändert 2'598 Zeilen. Erwartung: der Umsatz erscheint rückwirkend, sobald Frankreich bucht.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISS-004.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sales Database TR ES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Posting Date fehlt bei TR ES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Läuft</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ingo / Spanien</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Santi Gomez muss die alte 7-Tage-Version auf dem spanischen Server durch die neue 35-Tage-Version ersetzen, danach ist der laufende tägliche Import automatisch abgedeckt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SageSpainExportPackage/SageSpainFinalExportPackage/Export-SageSpainSalesCsv.ps1; Run-SpainRangeExportAndUpload-AllInOne.ps1; docs/FINANCE_ES_BUCHUNGSDATUM_2026-08-03.md Abschnitt 8, 9; Services/DatabaseSeedService.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19.08.2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Santi Gomez muss die neue Exportdatei auf dem spanischen Server ersetzen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NACHTRAG 19.08.2026: Backfill-Teil bestätigt behoben. App-seitige Spaltenzuordnung für PostingDate fehlte bei Spanien als einzigem Standort im Seed, nachgetragen über eine neue additive Funktion in Services/DatabaseSeedService.cs und am 18.08.2026 produktiv deployed, 534/534 Tests grün. Nach dem Deploy blieb PostingDate trotzdem bei 0 %, Ursache war NICHT ein Bedienfehler, sondern eine auf SharePoint nie aktualisierte CSV ohne PostingDate-Spalte. Korrigierte Datei per Tools/ManualImportUpload hochgeladen, alte Version vorher gesichert. Nach erneutem Reimport gegengemessen: PostingDate jetzt bei 1'523 von 7'220 TRES-Zeilen gefüllt (21,1 %), vorher 0 %. STAND 17.08.2026, LIVE VERIFIZIERT in einer RDP-Sitzung auf dem spanischen Sage-Server: Der Join-Schlüssel CodigoEmpresa/Ejercicio/Serie/Factura ist KORREKT, 53 von 53 Treffern (100 %) auf dem bereits gebuchten Fenster 23. bis 30.07. Die frühere Aussage in dieser Zeile, belegt sei nur die Syntax und Trefferquote sowie Schlüsselrichtigkeit seien offen, ist damit überholt. Die SQL selektiert FacturasTB.FechaAsiento als PostingDate und FacturasTB.Asiento als PostingDocument, per OUTER APPLY mit TOP 1 statt JOIN, weil 70 von 3'642 Rechnungsschlüsseln mehrere Buchungszeilen haben und ein JOIN die Verkaufszeilen vervielfacht hätte. Die im Testlauf 10. bis 13.08. leeren PostingDate-Werte lagen NICHT am Schlüssel, sondern an Buchungsverzug: das letzte gebuchte FechaFactura war der 30.07.2026. Deshalb ist das Zeitfenster des täglichen Delta-Laufs von 7 auf 35 Tage erweitert; die Anwendung dedupliziert über SourceLineId. Ebenfalls behoben: Resolve-RcloneExecutable nutzte $MyInvocation.MyCommand.Path innerhalb einer Funktion und damit zuverlässig $null, jetzt $PSScriptRoot. Diagnosewerkzeug: Analyze-SpainPostingDateKey.ps1 (read-only). Beim ersten Lauf in Spanien trotzdem die Zeilenzahl gegen den Vorlauf prüfen. Nebenbefund: die Paket-Zip war seit dem rclone-Fix veraltet und wurde neu gebaut. STATUS KORRIGIERT: stand als "Warten auf andere". Sage HAT das Buchungsdatum, es heisst FacturasTB.FechaAsiento und ist in der Stichprobe zu 100 % gefüllt; es fehlt nur im Export, und der Export ist unser. Offen ist nach der Live-Verifikation nur noch die Behandlung von Gutschriften. Am 12.08.2026 gemessen: PostingDate fehlt bei 5'731 von 5'731 ES-Zeilen. WICHTIGE KORREKTUR gegenüber der Analyse vom 28.07.: die 250 ES-Zeilen ohne jedes Datum fallen NICHT aus der Auswertung, sie sind schlechter eingeordnet. Die Spalte Finance | Date nutzt die Fallback-Kette bis zum ExtractionDate, deshalb landen sie im Monat des Exportlaufs. Nachgerechnet: ES hat im August nach Belegdatum 86 Zeilen, im Export 336, Differenz genau 250; UK 91 gegenüber 107, Differenz genau 16. Der laufende Monat wird also um 266 Zeilen aufgebläht.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISS-003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sales Database</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Der Lieferant wird bei sehr vielen Gesellschaften nicht angezeigt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>läuft</x:t>
+  </x:si>
+  <x:si>
+    <x:t>App / Standorte</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Technik ist fertig. Offen sind nur noch die Rohdatenquellen für DE und ES sowie Andreas' Entscheid zur CH/AT-Herstellerregel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>docs/SUPPLIER_LAENDERSTATUS_CH_AT_PRUEFUNG_2026-08-11.md; Services/GroupMarginSupplierClassifier.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Auf all8.xlsx vom 12.08.2026 gemessen: 18'263 von 97'537 Zeilen (18,7 %) haben alle drei Lieferantenfelder, 79'274 keines. Je Land UK 100 %, IT 71,2 %, IN 11,8 %, FR 5,2 %, US 0,4 %, CH/AT/DE/ES 0 %. Der Anteil ist gegenüber dem 11.08. leicht gesunken, weil der CH/AT-Nachlauf 1'183 Zeilen ohne Lieferantenfelder brachte; absolut hat sich nichts verschlechtert. NEU seit dem alten Kommentar: der technische Ersatz ist in beiden Stufen produktiv, MARC-Werk-1100-Fallback am 11.08. und Andreas' lokale Standardkosten bei sicherem Nichttreffer am 12.08. um 10:23. Wirkung nachgemessen: 22'950 Kandidaten, davon 10'817 CH-intern und 12'023 Lokal, 6'749 davon mit positivem Standardpreis. Indien ist über Sales Type zu 94,1 % klassifizierbar, nicht erneut zur Lieferantenpflege auffordern. CH/AT bleibt keine Zirkularreferenz.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISS-004.3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Customer Country code is not standardized</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Services/TransformationStrategies.cs, NormalizeCountryCodeTransformationStrategy</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Am 12.08.2026 dreifach belegt: der Typ NormalizeCountryCodeTransformationStrategy ist in der ausgelieferten Server-DLL nachgewiesen, die Produktivdaten zeigen für Spanien ISO-2-Codes (ES 3'955, BR 244, PT 233, PE 202, MX 195), und der Spaltenscan über all8.xlsx findet bei keinem Standort einen Wert, der nicht zweistellig ist. Der Reimport hat also stattgefunden. Die Dokumentation führte diesen Punkt noch als "Deploy offen", dein Blatt war hier besser als die MDs.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISS-003.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lieferant / lokale Standardkosten</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5'274 lokale Zeilen ohne positiven lokalen Standardpreis</x:t>
+  </x:si>
+  <x:si>
     <x:t>Offen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mittel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Range-Export 01.01.2026 bis 27.05.2026 nachziehen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SageSpainExportPackage/; Spain_Sales_range_20260528_to_20260603.csv</x:t>
-  </x:si>
-  <x:si>
-    <x:t>28.07.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>STATUS KORRIGIERT: stand als "Warten auf andere" mit Mail an Rohail. Es muss aber niemand antworten, denn die Sage-Export-SQL ist unsere und liegt in SageSpainExportPackage. Owner ist damit Ingo. Am 12.08.2026 unverändert bestätigt: Januar bis April 0 Zeilen, Mai nur 35, danach normal mit Juni 542 und Juli 503. 2025 ist über alle zwölf Monate vollständig.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISS-001</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TR AT und CH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Daten scheinen ab Mitte April nur noch vereinzelt geladen zu werden</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Beim nächsten Monatswechsel einmal gegenprüfen, dass der SAP-Batchjob weiterhin läuft</x:t>
-  </x:si>
-  <x:si>
-    <x:t>.tmp_tools/OdataProbe; docs/FINANCE_CHAT_2026_LUECKE_ROOTCAUSE_2026-07-28.md</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Zwei Stufen, beide erledigt. Erstens die Ursache von Juli: das Dashboard las das TEST-System T76 statt P76; Sites.SapServiceUrl steht inzwischen auf travp762, damit ist auch der frühere Punkt "Quelle umstellen" durch, und 2025 ist mit 30'642 Zeilen in beiden Systemen vollständig. Zweitens ein Folgeproblem, das darunter lag und im alten Log fehlte: von 31.07. bis 12.08. kamen für AT und CH KEINE neuen Zeilen, weil der SAP-Report Z_TRAFAG_DACH_EXPORT nur manuell lief. Ingo hat den Batchjob ZSCHWEIZ am 12.08.2026 auf täglich gestellt, und der Gesamtexport all8.xlsx von 14:39 belegt die Wirkung am selben Tag: CH 48'276 statt 47'142 Zeilen, AT 1'839 statt 1'790, August 2026 erstmals vorhanden, letzter Beleg 12.08. Der Wert liegt im vorher berechneten Fenster, 2025 ist erhalten und 2026 wurde ersetzt statt verdoppelt.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISS-001.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Datenzufluss TR FR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>B1 Frankreich enthält seit dem 30.07.2026 keine Rechnung mehr</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Warten auf andere</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Frankreich / Ingo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Frankreich gezielt fragen, warum seit dem 30.07. weder geliefert noch fakturiert wird, obwohl Aufträge und Wareneingänge weiterlaufen, und wann der Rückstand nachgebucht wird</x:t>
-  </x:si>
-  <x:si>
-    <x:t>.tmp_tools/HanaQ gegen FR01_P mit OINV, ORIN, ODLN, ORDR, ODRF (read-only, 12.08.2026)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Antwort aus Frankreich</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NEU AUFGENOMMEN, im alten Log nicht enthalten. Direkt in der Quelle geprüft: Rechnungen OINV letzter 30.07., Lieferscheine ODLN letzter 30.07., Gutschriften ORIN keine seit dem 25.07., Aufträge ORDR letzter 07.08., Entwürfe ODRF 12 Stück am 11.08. und alle vom Typ 20, also Wareneingänge zu Bestellungen. Frankreich arbeitet also weiter, nimmt Aufträge an und empfängt Ware, liefert und fakturiert aber nicht. Warenausgang und Faktura enden am exakt selben Tag, das deutet auf eine Betriebsschliessung oder eine Sperre im Ausgangsprozess, nicht auf ein Systemproblem. Saisonalität allein erklärt es nicht, im August 2025 gab es 99 Zeilen. Eine zweite Firmendatenbank aus dem B1-Upgrade ist ausgeschlossen, SYS.SCHEMAS kennt nur FR01_P. Die täglich frischen TRFR-Dateien in SharePoint sind UNSERE Exportausgaben, keine Lieferung aus Frankreich, und enthalten unverändert 2'598 Zeilen. Erwartung: der Umsatz erscheint rückwirkend, sobald Frankreich bucht.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISS-004.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sales Database TR ES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Posting Date fehlt bei TR ES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Läuft</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ingo / Spanien</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Paket auf den spanischen Sage-Server kopieren, Export einmal laufen lassen und dabei die Zeilenzahl gegen den Vorlauf prüfen, danach PostingDate beim Standort Spanien zuordnen und reimportieren</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SageSpainExportPackage/SageSpainFinalExportPackage/Export-SageSpainSalesCsv.ps1; Run-SpainRangeExportAndUpload-AllInOne.ps1; docs/FINANCE_ES_BUCHUNGSDATUM_2026-08-03.md Abschnitt 8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>17.08.2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RDP-Sitzung auf dem spanischen Sage-Server; Join-Schlüssel bis zur Messung eine Annahme</x:t>
-  </x:si>
-  <x:si>
-    <x:t>STAND 17.08.2026: das Feld ist im Exportskript EINGEBAUT und wartet nur noch auf den Lauf in Spanien. Die SQL selektiert FacturasTB.FechaAsiento als PostingDate und FacturasTB.Asiento als PostingDocument, per OUTER APPLY mit TOP 1 statt JOIN, weil 70 von 3'642 Rechnungsschlüsseln mehrere Buchungszeilen haben und ein JOIN die Verkaufszeilen vervielfacht hätte. Belegt ist bisher NUR die Syntax (ScriptDom, alle vier Varianten, mit Gegenprobe); Trefferquote, Schlüsselrichtigkeit und Gutschriften sind offen. Beim ersten Lauf zwingend die Zeilenzahl gegen den Vorlauf prüfen. Nebenbefund: die Paket-Zip war seit dem rclone-Fix veraltet und wurde neu gebaut. STATUS KORRIGIERT: stand als "Warten auf andere". Sage HAT das Buchungsdatum, es heisst FacturasTB.FechaAsiento und ist in der Stichprobe zu 100 % gefüllt; es fehlt nur im Export, und der Export ist unser. Offen sind der Join-Schlüssel und die Behandlung von Gutschriften. Am 12.08.2026 gemessen: PostingDate fehlt bei 5'731 von 5'731 ES-Zeilen. WICHTIGE KORREKTUR gegenüber der Analyse vom 28.07.: die 250 ES-Zeilen ohne jedes Datum fallen NICHT aus der Auswertung, sie sind schlechter eingeordnet. Die Spalte Finance | Date nutzt die Fallback-Kette bis zum ExtractionDate, deshalb landen sie im Monat des Exportlaufs. Nachgerechnet: ES hat im August nach Belegdatum 86 Zeilen, im Export 336, Differenz genau 250; UK 91 gegenüber 107, Differenz genau 16. Der laufende Monat wird also um 266 Zeilen aufgebläht.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISS-003</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sales Database</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Der Lieferant wird bei sehr vielen Gesellschaften nicht angezeigt</x:t>
-  </x:si>
-  <x:si>
-    <x:t>läuft</x:t>
-  </x:si>
-  <x:si>
-    <x:t>App / Standorte</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Technik ist fertig. Offen sind nur noch die Rohdatenquellen für DE und ES sowie Andreas' Entscheid zur CH/AT-Herstellerregel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>docs/SUPPLIER_LAENDERSTATUS_CH_AT_PRUEFUNG_2026-08-11.md; Services/GroupMarginSupplierClassifier.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Auf all8.xlsx vom 12.08.2026 gemessen: 18'263 von 97'537 Zeilen (18,7 %) haben alle drei Lieferantenfelder, 79'274 keines. Je Land UK 100 %, IT 71,2 %, IN 11,8 %, FR 5,2 %, US 0,4 %, CH/AT/DE/ES 0 %. Der Anteil ist gegenüber dem 11.08. leicht gesunken, weil der CH/AT-Nachlauf 1'183 Zeilen ohne Lieferantenfelder brachte; absolut hat sich nichts verschlechtert. NEU seit dem alten Kommentar: der technische Ersatz ist in beiden Stufen produktiv, MARC-Werk-1100-Fallback am 11.08. und Andreas' lokale Standardkosten bei sicherem Nichttreffer am 12.08. um 10:23. Wirkung nachgemessen: 22'950 Kandidaten, davon 10'817 CH-intern und 12'023 Lokal, 6'749 davon mit positivem Standardpreis. Indien ist über Sales Type zu 94,1 % klassifizierbar, nicht erneut zur Lieferantenpflege auffordern. CH/AT bleibt keine Zirkularreferenz.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISS-004.3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Customer Country code is not standardized</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Services/TransformationStrategies.cs, NormalizeCountryCodeTransformationStrategy</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Am 12.08.2026 dreifach belegt: der Typ NormalizeCountryCodeTransformationStrategy ist in der ausgelieferten Server-DLL nachgewiesen, die Produktivdaten zeigen für Spanien ISO-2-Codes (ES 3'955, BR 244, PT 233, PE 202, MX 195), und der Spaltenscan über all8.xlsx findet bei keinem Standort einen Wert, der nicht zweistellig ist. Der Reimport hat also stattgefunden. Die Dokumentation führte diesen Punkt noch als "Deploy offen", dein Blatt war hier besser als die MDs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISS-003.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lieferant / lokale Standardkosten</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5'274 lokale Zeilen ohne positiven lokalen Standardpreis</x:t>
   </x:si>
   <x:si>
     <x:t>Standorte</x:t>
@@ -1317,29 +1320,29 @@
       <x:c r="D4" s="9" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="E4" s="10" t="s">
+      <x:c r="E4" s="5" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F4" s="7" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="F4" s="7" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="G4" s="7" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="H4" s="9" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="I4" s="9" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="I4" s="9" t="s">
+      <x:c r="J4" s="7" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="J4" s="7" t="s">
+      <x:c r="K4" s="7" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L4" s="7" t="s">
         <x:v>41</x:v>
-      </x:c>
-      <x:c r="K4" s="7" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L4" s="7" t="s">
-        <x:v>24</x:v>
       </x:c>
       <x:c r="M4" s="9" t="s">
         <x:v>23</x:v>
@@ -1377,7 +1380,7 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="J5" s="2" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K5" s="2" t="s">
         <x:v>23</x:v>
@@ -1453,7 +1456,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="F7" s="7" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G7" s="7" t="s">
         <x:v>62</x:v>
@@ -1465,7 +1468,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="J7" s="7" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K7" s="7" t="s">
         <x:v>23</x:v>
@@ -1509,7 +1512,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="J8" s="2" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K8" s="2" t="s">
         <x:v>23</x:v>
@@ -1541,7 +1544,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
         <x:v>29</x:v>
@@ -1553,7 +1556,7 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="J9" s="7" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K9" s="7" t="s">
         <x:v>23</x:v>
@@ -1582,19 +1585,19 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="E10" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F10" s="7" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F10" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="H10" s="9" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="I10" s="9" t="s">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="J10" s="7" t="s">
         <x:v>24</x:v>
@@ -1609,7 +1612,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N10" s="9" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:14">
@@ -1617,31 +1620,31 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B11" s="8" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="C11" s="9" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D11" s="9" t="s">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E11" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F11" s="7" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>90</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="H11" s="9" t="s">
-        <x:v>91</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="I11" s="9" t="s">
-        <x:v>92</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="J11" s="7" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="K11" s="7" t="s">
         <x:v>23</x:v>
@@ -1650,10 +1653,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="M11" s="9" t="s">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="N11" s="9" t="s">
-        <x:v>94</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:14">
@@ -1661,28 +1664,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B12" s="8" t="s">
-        <x:v>95</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C12" s="9" t="s">
-        <x:v>96</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D12" s="9" t="s">
-        <x:v>97</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E12" s="13" t="s">
-        <x:v>98</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="F12" s="11" t="s">
         <x:v>18</x:v>
       </x:c>
       <x:c r="G12" s="7" t="s">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H12" s="9" t="s">
-        <x:v>100</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="I12" s="9" t="s">
-        <x:v>101</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="J12" s="7" t="s">
         <x:v>32</x:v>
@@ -1694,10 +1697,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="M12" s="9" t="s">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="N12" s="9" t="s">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:14">
@@ -1705,28 +1708,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="8" t="s">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C13" s="9" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D13" s="9" t="s">
-        <x:v>106</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E13" s="13" t="s">
-        <x:v>107</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F13" s="7" t="s">
-        <x:v>108</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="G13" s="7" t="s">
-        <x:v>109</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="H13" s="9" t="s">
-        <x:v>110</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="I13" s="9" t="s">
-        <x:v>111</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="J13" s="7" t="s">
         <x:v>24</x:v>
@@ -1738,10 +1741,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="M13" s="9" t="s">
-        <x:v>112</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="N13" s="9" t="s">
-        <x:v>113</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:14">
@@ -1749,28 +1752,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
-        <x:v>114</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C14" s="4" t="s">
-        <x:v>115</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D14" s="4" t="s">
-        <x:v>116</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E14" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="F14" s="2" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="G14" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
       <x:c r="H14" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="I14" s="4" t="s">
-        <x:v>118</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="J14" s="2" t="s">
         <x:v>24</x:v>
@@ -1785,7 +1788,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N14" s="4" t="s">
-        <x:v>119</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:14">
@@ -1793,31 +1796,31 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
-        <x:v>120</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="C15" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D15" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E15" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F15" s="2" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="G15" s="2" t="s">
-        <x:v>123</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="H15" s="4" t="s">
-        <x:v>124</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="I15" s="4" t="s">
-        <x:v>125</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="J15" s="2" t="s">
-        <x:v>126</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="K15" s="2" t="s">
         <x:v>23</x:v>
@@ -1826,10 +1829,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="M15" s="4" t="s">
-        <x:v>127</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="N15" s="4" t="s">
-        <x:v>128</x:v>
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:14">
@@ -1837,28 +1840,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="C16" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="D16" s="4" t="s">
-        <x:v>131</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E16" s="12" t="s">
         <x:v>71</x:v>
       </x:c>
       <x:c r="F16" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G16" s="2" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="H16" s="4" t="s">
-        <x:v>132</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="I16" s="4" t="s">
-        <x:v>133</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="J16" s="2" t="s">
         <x:v>22</x:v>
@@ -1873,7 +1876,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N16" s="4" t="s">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:14">
@@ -1881,34 +1884,34 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="8" t="s">
-        <x:v>135</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C17" s="9" t="s">
-        <x:v>136</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="D17" s="9" t="s">
-        <x:v>137</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E17" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F17" s="7" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>138</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="H17" s="9" t="s">
-        <x:v>139</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="I17" s="9" t="s">
-        <x:v>140</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="J17" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="K17" s="7" t="s">
-        <x:v>142</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="L17" s="7" t="s">
         <x:v>24</x:v>
@@ -1917,7 +1920,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="N17" s="9" t="s">
-        <x:v>143</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:14">
@@ -1925,31 +1928,31 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
-        <x:v>144</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="C18" s="4" t="s">
-        <x:v>145</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D18" s="4" t="s">
-        <x:v>146</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="E18" s="10" t="s">
-        <x:v>37</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="F18" s="2" t="s">
-        <x:v>108</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="G18" s="2" t="s">
-        <x:v>147</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="H18" s="4" t="s">
-        <x:v>148</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="I18" s="4" t="s">
-        <x:v>149</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="J18" s="2" t="s">
-        <x:v>150</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="K18" s="2" t="s">
         <x:v>23</x:v>
@@ -1958,10 +1961,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="M18" s="4" t="s">
-        <x:v>151</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="N18" s="4" t="s">
-        <x:v>152</x:v>
+        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:14">
@@ -1969,31 +1972,31 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C19" s="4" t="s">
-        <x:v>154</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D19" s="4" t="s">
-        <x:v>155</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="E19" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F19" s="2" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="G19" s="2" t="s">
-        <x:v>156</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="H19" s="4" t="s">
-        <x:v>157</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="I19" s="4" t="s">
-        <x:v>158</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="J19" s="2" t="s">
-        <x:v>159</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="K19" s="2" t="s">
         <x:v>23</x:v>
@@ -2002,10 +2005,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="M19" s="4" t="s">
-        <x:v>160</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="N19" s="4" t="s">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:14">
@@ -2013,43 +2016,43 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C20" s="4" t="s">
-        <x:v>163</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D20" s="4" t="s">
-        <x:v>164</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="E20" s="10" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F20" s="2" t="s">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="G20" s="2" t="s">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H20" s="4" t="s">
-        <x:v>165</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="I20" s="4" t="s">
-        <x:v>166</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="J20" s="2" t="s">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="K20" s="2" t="s">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L20" s="2" t="s">
-        <x:v>167</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="M20" s="4" t="s">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="N20" s="4" t="s">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2076,82 +2079,82 @@
   <x:sheetData>
     <x:row r="1" spans="1:2">
       <x:c r="A1" s="15" t="s">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B1" s="16" t="s">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:2" ht="46" customHeight="1">
       <x:c r="A2" s="17" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B2" s="14" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:2" ht="46" customHeight="1">
       <x:c r="A3" s="17" t="s">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B3" s="14" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:2" ht="46" customHeight="1">
       <x:c r="A4" s="17" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B4" s="14" t="s">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:2" ht="46" customHeight="1">
       <x:c r="A5" s="17" t="s">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B5" s="14" t="s">
-        <x:v>179</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:2" ht="46" customHeight="1">
       <x:c r="A6" s="17" t="s">
-        <x:v>180</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B6" s="14" t="s">
-        <x:v>181</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:2" ht="46" customHeight="1">
       <x:c r="A7" s="17" t="s">
-        <x:v>182</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B7" s="14" t="s">
-        <x:v>183</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:2" ht="46" customHeight="1">
       <x:c r="A8" s="17" t="s">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B8" s="14" t="s">
-        <x:v>185</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:2" ht="46" customHeight="1">
       <x:c r="A9" s="17" t="s">
-        <x:v>186</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B9" s="14" t="s">
-        <x:v>187</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:2" ht="46" customHeight="1">
       <x:c r="A10" s="17" t="s">
-        <x:v>188</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B10" s="14" t="s">
-        <x:v>189</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>